<commit_message>
feat(competitor-intel): tidy Gmail newsletters into a Notion competitor/inspiration DB
Weekly cron reads yourhavenpilates@gmail.com (separate OAuth from Calendar,
gmail.modify scope): tags+archives newsletters from a founder-maintained
Notion source list, then extracts events/promotions/positioning/product
findings with Claude Haiku and writes them to a new Competitor Intel DB.
Categoria is left for the founder to set by hand. Gmail labels double as
the only run-to-run state (no separate checkpoint file). Includes a
one-off backfill script for the existing tagged backlog, a dry-run flag,
and /auth_gmail for the founder-DM OAuth flow.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/notion-db-config.xlsx
+++ b/docs/notion-db-config.xlsx
@@ -14,6 +14,8 @@
     <sheet name="Eventos" sheetId="9" r:id="rId9"/>
     <sheet name="Listas" sheetId="10" r:id="rId10"/>
     <sheet name="Founder Focus" sheetId="11" r:id="rId11"/>
+    <sheet name="Fontes Conc-Inspo" sheetId="12" r:id="rId12"/>
+    <sheet name="Competitor Intel" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -890,6 +892,236 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Propriedade</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Valores possíveis</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Notas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nome</v>
+      </c>
+      <c r="B2" t="str">
+        <v>title</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Email/Domínio</v>
+      </c>
+      <c r="B3" t="str">
+        <v>text</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>remetente/domínio que o cron usa para encontrar newsletters na Inbox</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Categoria</v>
+      </c>
+      <c r="B4" t="str">
+        <v>select</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Concorrência | Inspiração</v>
+      </c>
+      <c r="D4" t="str">
+        <v>referência do founder — não é copiado para o Competitor Intel</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Ativo</v>
+      </c>
+      <c r="B5" t="str">
+        <v>checkbox</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>desmarcar pausa a fonte sem apagar a linha</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Propriedade</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Valores possíveis</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Notas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nome</v>
+      </c>
+      <c r="B2" t="str">
+        <v>title</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>gerado pelo bot a partir do resumo</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Fonte</v>
+      </c>
+      <c r="B3" t="str">
+        <v>text</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>nome do remetente</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Categoria</v>
+      </c>
+      <c r="B4" t="str">
+        <v>select</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Concorrência | Inspiração</v>
+      </c>
+      <c r="D4" t="str">
+        <v>deixado por preencher pelo bot — o founder classifica à mão</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="B5" t="str">
+        <v>multi_select</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>cria automaticamente novos valores — Evento, Promoção/Campanha, Posicionamento/Mensagem, Produto/Serviço, ou outros propostos pelo extrator</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Resumo</v>
+      </c>
+      <c r="B6" t="str">
+        <v>text</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Data do email</v>
+      </c>
+      <c r="B7" t="str">
+        <v>date</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Assunto do email</v>
+      </c>
+      <c r="B8" t="str">
+        <v>text</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Link Gmail</v>
+      </c>
+      <c r="B9" t="str">
+        <v>url</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>link direto para o email de origem, mesmo depois de arquivado</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D13"/>

</xml_diff>

<commit_message>
feat(competitor-intel): tidy Gmail newsletters into a Notion competitor/inspiration DB (#12)
Weekly cron reads yourhavenpilates@gmail.com (separate OAuth from Calendar,
gmail.modify scope): tags+archives newsletters from a founder-maintained
Notion source list, then extracts events/promotions/positioning/product
findings with Claude Haiku and writes them to a new Competitor Intel DB.
Categoria is left for the founder to set by hand. Gmail labels double as
the only run-to-run state (no separate checkpoint file). Includes a
one-off backfill script for the existing tagged backlog, a dry-run flag,
and /auth_gmail for the founder-DM OAuth flow.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/notion-db-config.xlsx
+++ b/docs/notion-db-config.xlsx
@@ -14,6 +14,8 @@
     <sheet name="Eventos" sheetId="9" r:id="rId9"/>
     <sheet name="Listas" sheetId="10" r:id="rId10"/>
     <sheet name="Founder Focus" sheetId="11" r:id="rId11"/>
+    <sheet name="Fontes Conc-Inspo" sheetId="12" r:id="rId12"/>
+    <sheet name="Competitor Intel" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -890,6 +892,236 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Propriedade</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Valores possíveis</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Notas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nome</v>
+      </c>
+      <c r="B2" t="str">
+        <v>title</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Email/Domínio</v>
+      </c>
+      <c r="B3" t="str">
+        <v>text</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>remetente/domínio que o cron usa para encontrar newsletters na Inbox</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Categoria</v>
+      </c>
+      <c r="B4" t="str">
+        <v>select</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Concorrência | Inspiração</v>
+      </c>
+      <c r="D4" t="str">
+        <v>referência do founder — não é copiado para o Competitor Intel</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Ativo</v>
+      </c>
+      <c r="B5" t="str">
+        <v>checkbox</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>desmarcar pausa a fonte sem apagar a linha</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Propriedade</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Valores possíveis</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Notas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nome</v>
+      </c>
+      <c r="B2" t="str">
+        <v>title</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>gerado pelo bot a partir do resumo</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Fonte</v>
+      </c>
+      <c r="B3" t="str">
+        <v>text</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>nome do remetente</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Categoria</v>
+      </c>
+      <c r="B4" t="str">
+        <v>select</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Concorrência | Inspiração</v>
+      </c>
+      <c r="D4" t="str">
+        <v>deixado por preencher pelo bot — o founder classifica à mão</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="B5" t="str">
+        <v>multi_select</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>cria automaticamente novos valores — Evento, Promoção/Campanha, Posicionamento/Mensagem, Produto/Serviço, ou outros propostos pelo extrator</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Resumo</v>
+      </c>
+      <c r="B6" t="str">
+        <v>text</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Data do email</v>
+      </c>
+      <c r="B7" t="str">
+        <v>date</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Assunto do email</v>
+      </c>
+      <c r="B8" t="str">
+        <v>text</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Link Gmail</v>
+      </c>
+      <c r="B9" t="str">
+        <v>url</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>link direto para o email de origem, mesmo depois de arquivado</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D13"/>

</xml_diff>